<commit_message>
MAJ liste activites Sprint 1 - toutes les issues
</commit_message>
<xml_diff>
--- a/docs/TP2-FoxTrot-Liste_Activites-Sprint1.xlsx
+++ b/docs/TP2-FoxTrot-Liste_Activites-Sprint1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UQAM\Été 2026\INF6150 (Génie logiciel - Conduite de projets informatiques)\Travaux Pratiques\TP2\fixmycar\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BC39A44-B1DA-46CA-BF0A-825A7C3568EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3965BC-C517-42C9-8312-A796A0F5731C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-135" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Activités" sheetId="1" r:id="rId1"/>
@@ -1181,7 +1181,7 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="225">
+  <cellXfs count="221">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1780,6 +1780,19 @@
     <xf numFmtId="166" fontId="28" fillId="0" borderId="8" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="16" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="16" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1822,31 +1835,12 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="16" fontId="17" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="16" fillId="14" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="16" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Monétaire" xfId="1" builtinId="4"/>
@@ -2544,120 +2538,120 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="204" t="s">
+      <c r="B1" s="209" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
-      <c r="F1" s="204"/>
-      <c r="G1" s="204"/>
-      <c r="H1" s="204"/>
-      <c r="I1" s="204"/>
-      <c r="J1" s="204"/>
-      <c r="K1" s="204"/>
+      <c r="C1" s="209"/>
+      <c r="D1" s="209"/>
+      <c r="E1" s="209"/>
+      <c r="F1" s="209"/>
+      <c r="G1" s="209"/>
+      <c r="H1" s="209"/>
+      <c r="I1" s="209"/>
+      <c r="J1" s="209"/>
+      <c r="K1" s="209"/>
       <c r="L1" s="11"/>
-      <c r="M1" s="206" t="s">
+      <c r="M1" s="211" t="s">
         <v>1</v>
       </c>
-      <c r="N1" s="206"/>
-      <c r="O1" s="206"/>
-      <c r="P1" s="206"/>
-      <c r="Q1" s="206"/>
-      <c r="R1" s="206"/>
-      <c r="S1" s="206"/>
-      <c r="T1" s="206"/>
-      <c r="U1" s="206"/>
-      <c r="V1" s="206"/>
-      <c r="W1" s="206"/>
-      <c r="X1" s="206"/>
-      <c r="Y1" s="206"/>
-      <c r="Z1" s="206"/>
-      <c r="AA1" s="206"/>
-      <c r="AB1" s="206"/>
-      <c r="AC1" s="206"/>
+      <c r="N1" s="211"/>
+      <c r="O1" s="211"/>
+      <c r="P1" s="211"/>
+      <c r="Q1" s="211"/>
+      <c r="R1" s="211"/>
+      <c r="S1" s="211"/>
+      <c r="T1" s="211"/>
+      <c r="U1" s="211"/>
+      <c r="V1" s="211"/>
+      <c r="W1" s="211"/>
+      <c r="X1" s="211"/>
+      <c r="Y1" s="211"/>
+      <c r="Z1" s="211"/>
+      <c r="AA1" s="211"/>
+      <c r="AB1" s="211"/>
+      <c r="AC1" s="211"/>
     </row>
     <row r="2" spans="1:43" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="217" t="s">
+      <c r="B2" s="203" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="217"/>
-      <c r="D2" s="217"/>
-      <c r="E2" s="217"/>
-      <c r="F2" s="217"/>
-      <c r="G2" s="217"/>
-      <c r="H2" s="217"/>
-      <c r="I2" s="217"/>
-      <c r="J2" s="217"/>
-      <c r="K2" s="217"/>
+      <c r="C2" s="203"/>
+      <c r="D2" s="203"/>
+      <c r="E2" s="203"/>
+      <c r="F2" s="203"/>
+      <c r="G2" s="203"/>
+      <c r="H2" s="203"/>
+      <c r="I2" s="203"/>
+      <c r="J2" s="203"/>
+      <c r="K2" s="203"/>
       <c r="L2" s="54"/>
-      <c r="M2" s="205" t="s">
+      <c r="M2" s="210" t="s">
         <v>3</v>
       </c>
-      <c r="N2" s="205"/>
-      <c r="O2" s="205"/>
-      <c r="P2" s="205"/>
-      <c r="Q2" s="205"/>
-      <c r="R2" s="205"/>
-      <c r="S2" s="205"/>
-      <c r="T2" s="205"/>
-      <c r="U2" s="205"/>
-      <c r="V2" s="205"/>
-      <c r="W2" s="205"/>
-      <c r="X2" s="205"/>
-      <c r="Y2" s="205"/>
-      <c r="Z2" s="205"/>
-      <c r="AA2" s="205"/>
-      <c r="AB2" s="205"/>
-      <c r="AC2" s="205"/>
+      <c r="N2" s="210"/>
+      <c r="O2" s="210"/>
+      <c r="P2" s="210"/>
+      <c r="Q2" s="210"/>
+      <c r="R2" s="210"/>
+      <c r="S2" s="210"/>
+      <c r="T2" s="210"/>
+      <c r="U2" s="210"/>
+      <c r="V2" s="210"/>
+      <c r="W2" s="210"/>
+      <c r="X2" s="210"/>
+      <c r="Y2" s="210"/>
+      <c r="Z2" s="210"/>
+      <c r="AA2" s="210"/>
+      <c r="AB2" s="210"/>
+      <c r="AC2" s="210"/>
       <c r="AF2" s="148"/>
       <c r="AG2" s="148"/>
       <c r="AH2" s="148"/>
     </row>
     <row r="3" spans="1:43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="210" t="s">
+      <c r="B3" s="215" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="211"/>
+      <c r="C3" s="216"/>
       <c r="D3" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="212" t="s">
+      <c r="E3" s="217" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="213"/>
-      <c r="G3" s="213"/>
-      <c r="H3" s="213"/>
-      <c r="I3" s="213"/>
-      <c r="J3" s="213"/>
+      <c r="F3" s="218"/>
+      <c r="G3" s="218"/>
+      <c r="H3" s="218"/>
+      <c r="I3" s="218"/>
+      <c r="J3" s="218"/>
       <c r="K3" s="74" t="s">
         <v>7</v>
       </c>
       <c r="L3" s="12"/>
-      <c r="M3" s="214" t="s">
+      <c r="M3" s="202" t="s">
         <v>4</v>
       </c>
-      <c r="N3" s="214"/>
+      <c r="N3" s="202"/>
       <c r="O3" s="141" t="s">
         <v>5</v>
       </c>
-      <c r="P3" s="214" t="s">
+      <c r="P3" s="202" t="s">
         <v>6</v>
       </c>
-      <c r="Q3" s="214"/>
-      <c r="R3" s="214"/>
-      <c r="S3" s="214"/>
-      <c r="T3" s="214"/>
-      <c r="U3" s="214"/>
-      <c r="V3" s="214"/>
-      <c r="W3" s="214"/>
-      <c r="X3" s="214"/>
-      <c r="Y3" s="214"/>
-      <c r="Z3" s="214" t="s">
+      <c r="Q3" s="202"/>
+      <c r="R3" s="202"/>
+      <c r="S3" s="202"/>
+      <c r="T3" s="202"/>
+      <c r="U3" s="202"/>
+      <c r="V3" s="202"/>
+      <c r="W3" s="202"/>
+      <c r="X3" s="202"/>
+      <c r="Y3" s="202"/>
+      <c r="Z3" s="202" t="s">
         <v>8</v>
       </c>
-      <c r="AA3" s="214"/>
-      <c r="AB3" s="214"/>
+      <c r="AA3" s="202"/>
+      <c r="AB3" s="202"/>
       <c r="AC3" s="141" t="s">
         <v>9</v>
       </c>
@@ -2891,7 +2885,7 @@
         <f>AA6-K6</f>
         <v>0</v>
       </c>
-      <c r="AC6" s="207"/>
+      <c r="AC6" s="212"/>
       <c r="AE6" s="20" t="s">
         <v>34</v>
       </c>
@@ -2992,7 +2986,7 @@
         <f t="shared" ref="AB7:AB10" si="5">AA7-K7</f>
         <v>0</v>
       </c>
-      <c r="AC7" s="207"/>
+      <c r="AC7" s="212"/>
       <c r="AF7" s="55"/>
       <c r="AG7" s="55"/>
       <c r="AH7" s="55"/>
@@ -3090,7 +3084,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC8" s="207"/>
+      <c r="AC8" s="212"/>
       <c r="AE8" s="152" t="s">
         <v>37</v>
       </c>
@@ -3200,7 +3194,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC9" s="207"/>
+      <c r="AC9" s="212"/>
       <c r="AE9" s="152" t="s">
         <v>43</v>
       </c>
@@ -3312,7 +3306,7 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="AC10" s="207"/>
+      <c r="AC10" s="212"/>
       <c r="AE10" s="152" t="s">
         <v>46</v>
       </c>
@@ -3432,18 +3426,18 @@
         <f t="shared" ref="AB11" si="13">Z11-K11</f>
         <v>0</v>
       </c>
-      <c r="AC11" s="208"/>
+      <c r="AC11" s="213"/>
       <c r="AD11" s="37"/>
       <c r="AE11" s="155" t="s">
         <v>49</v>
       </c>
       <c r="AF11" s="156">
         <f>U37</f>
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="AG11" s="162">
         <f>Z37</f>
-        <v>1430</v>
+        <v>5720</v>
       </c>
       <c r="AH11" s="157">
         <v>9</v>
@@ -3473,8 +3467,8 @@
       <c r="J12" s="114"/>
       <c r="K12" s="68"/>
       <c r="L12" s="29"/>
-      <c r="M12" s="215"/>
-      <c r="N12" s="215"/>
+      <c r="M12" s="219"/>
+      <c r="N12" s="219"/>
       <c r="O12" s="113"/>
       <c r="P12" s="113"/>
       <c r="Q12" s="113"/>
@@ -3598,17 +3592,17 @@
         <f t="shared" ref="AB13:AB17" si="20">Z13-K13</f>
         <v>0</v>
       </c>
-      <c r="AC13" s="209"/>
+      <c r="AC13" s="214"/>
       <c r="AE13" s="167" t="s">
         <v>53</v>
       </c>
       <c r="AF13" s="168">
         <f>U45</f>
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="AG13" s="169">
         <f>Z45</f>
-        <v>8910</v>
+        <v>13200</v>
       </c>
       <c r="AH13" s="170">
         <v>2</v>
@@ -3707,17 +3701,17 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC14" s="207"/>
+      <c r="AC14" s="212"/>
       <c r="AE14" s="152" t="s">
         <v>23</v>
       </c>
       <c r="AF14" s="154">
         <f>V45</f>
-        <v>257</v>
+        <v>218</v>
       </c>
       <c r="AG14" s="161">
         <f>V45*tarif</f>
-        <v>28270</v>
+        <v>23980</v>
       </c>
       <c r="AH14" s="153">
         <v>7</v>
@@ -3817,7 +3811,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC15" s="207"/>
+      <c r="AC15" s="212"/>
       <c r="AE15" s="171" t="s">
         <v>56</v>
       </c>
@@ -3928,7 +3922,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC16" s="207"/>
+      <c r="AC16" s="212"/>
       <c r="AE16" s="175" t="s">
         <v>57</v>
       </c>
@@ -4048,7 +4042,7 @@
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="AC17" s="208"/>
+      <c r="AC17" s="213"/>
       <c r="AD17" s="37"/>
       <c r="AE17" s="152" t="s">
         <v>59</v>
@@ -4065,7 +4059,7 @@
         <f>AH16-AH15</f>
         <v>0</v>
       </c>
-      <c r="AI17" s="200" t="s">
+      <c r="AI17" s="205" t="s">
         <v>60</v>
       </c>
       <c r="AJ17" s="37"/>
@@ -4092,8 +4086,8 @@
       <c r="J18" s="120"/>
       <c r="K18" s="76"/>
       <c r="L18" s="51"/>
-      <c r="M18" s="218"/>
-      <c r="N18" s="218"/>
+      <c r="M18" s="204"/>
+      <c r="N18" s="204"/>
       <c r="O18" s="138"/>
       <c r="P18" s="119"/>
       <c r="Q18" s="119"/>
@@ -4109,13 +4103,13 @@
       <c r="AA18" s="76"/>
       <c r="AB18" s="76"/>
       <c r="AC18" s="44"/>
-      <c r="AE18" s="202" t="s">
+      <c r="AE18" s="207" t="s">
         <v>62</v>
       </c>
-      <c r="AF18" s="202"/>
-      <c r="AG18" s="202"/>
-      <c r="AH18" s="202"/>
-      <c r="AI18" s="201"/>
+      <c r="AF18" s="207"/>
+      <c r="AG18" s="207"/>
+      <c r="AH18" s="207"/>
+      <c r="AI18" s="206"/>
     </row>
     <row r="19" spans="1:43" s="19" customFormat="1" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A19" s="187" t="s">
@@ -4190,7 +4184,7 @@
         <v>13</v>
       </c>
       <c r="X19" s="131" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="Y19" s="137">
         <f t="shared" ref="Y19:Y36" si="30">(W19-J19)</f>
@@ -4209,11 +4203,11 @@
         <v>0</v>
       </c>
       <c r="AC19" s="6"/>
-      <c r="AE19" s="203"/>
-      <c r="AF19" s="203"/>
-      <c r="AG19" s="203"/>
-      <c r="AH19" s="203"/>
-      <c r="AI19" s="201"/>
+      <c r="AE19" s="208"/>
+      <c r="AF19" s="208"/>
+      <c r="AG19" s="208"/>
+      <c r="AH19" s="208"/>
+      <c r="AI19" s="206"/>
     </row>
     <row r="20" spans="1:43" s="20" customFormat="1" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
@@ -4252,31 +4246,43 @@
         <v>1320</v>
       </c>
       <c r="L20" s="9"/>
-      <c r="M20" s="106"/>
+      <c r="M20" s="106">
+        <v>46210</v>
+      </c>
       <c r="N20" s="136">
         <f t="shared" si="27"/>
-        <v>-46194</v>
+        <v>16</v>
       </c>
       <c r="O20" s="142"/>
-      <c r="P20" s="131"/>
-      <c r="Q20" s="131"/>
-      <c r="R20" s="131"/>
-      <c r="S20" s="131"/>
-      <c r="T20" s="131"/>
+      <c r="P20" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q20" s="131">
+        <v>1</v>
+      </c>
+      <c r="R20" s="131">
+        <v>1</v>
+      </c>
+      <c r="S20" s="131">
+        <v>1</v>
+      </c>
+      <c r="T20" s="131">
+        <v>8</v>
+      </c>
       <c r="U20" s="137">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="V20" s="131">
         <f t="shared" ref="V20:V36" si="34">J20-U20</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="W20" s="137">
         <f t="shared" si="29"/>
         <v>12</v>
       </c>
       <c r="X20" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y20" s="137">
         <f t="shared" si="30"/>
@@ -4284,7 +4290,7 @@
       </c>
       <c r="Z20" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1320</v>
       </c>
       <c r="AA20" s="109">
         <f t="shared" si="32"/>
@@ -4292,7 +4298,7 @@
       </c>
       <c r="AB20" s="139">
         <f t="shared" ref="AB20:AB36" si="35">Z20-K20</f>
-        <v>-1320</v>
+        <v>0</v>
       </c>
       <c r="AC20" s="6"/>
       <c r="AD20" s="19"/>
@@ -4300,7 +4306,7 @@
       <c r="AF20" s="55"/>
       <c r="AG20" s="55"/>
       <c r="AH20" s="55"/>
-      <c r="AI20" s="201"/>
+      <c r="AI20" s="206"/>
     </row>
     <row r="21" spans="1:43" s="19" customFormat="1" ht="15.75" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
       <c r="A21" s="187" t="s">
@@ -4339,31 +4345,43 @@
         <v>1540</v>
       </c>
       <c r="L21" s="9"/>
-      <c r="M21" s="106"/>
+      <c r="M21" s="106">
+        <v>46210</v>
+      </c>
       <c r="N21" s="136">
         <f t="shared" si="27"/>
-        <v>-46194</v>
+        <v>16</v>
       </c>
       <c r="O21" s="142"/>
-      <c r="P21" s="131"/>
-      <c r="Q21" s="131"/>
-      <c r="R21" s="131"/>
-      <c r="S21" s="131"/>
-      <c r="T21" s="131"/>
+      <c r="P21" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q21" s="131">
+        <v>2</v>
+      </c>
+      <c r="R21" s="131">
+        <v>1</v>
+      </c>
+      <c r="S21" s="131">
+        <v>9</v>
+      </c>
+      <c r="T21" s="131">
+        <v>1</v>
+      </c>
       <c r="U21" s="137">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="V21" s="131">
         <f t="shared" si="34"/>
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="W21" s="137">
         <f t="shared" si="29"/>
         <v>14</v>
       </c>
       <c r="X21" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y21" s="137">
         <f t="shared" si="30"/>
@@ -4371,7 +4389,7 @@
       </c>
       <c r="Z21" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1540</v>
       </c>
       <c r="AA21" s="109">
         <f t="shared" si="32"/>
@@ -4379,7 +4397,7 @@
       </c>
       <c r="AB21" s="139">
         <f t="shared" si="35"/>
-        <v>-1540</v>
+        <v>0</v>
       </c>
       <c r="AC21" s="6"/>
       <c r="AF21" s="55"/>
@@ -4424,31 +4442,43 @@
         <v>1430</v>
       </c>
       <c r="L22" s="9"/>
-      <c r="M22" s="106"/>
+      <c r="M22" s="106">
+        <v>46209</v>
+      </c>
       <c r="N22" s="136">
         <f t="shared" si="27"/>
-        <v>-46194</v>
+        <v>15</v>
       </c>
       <c r="O22" s="142"/>
-      <c r="P22" s="131"/>
-      <c r="Q22" s="131"/>
-      <c r="R22" s="131"/>
-      <c r="S22" s="131"/>
-      <c r="T22" s="131"/>
+      <c r="P22" s="131">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="131">
+        <v>9</v>
+      </c>
+      <c r="R22" s="131">
+        <v>1</v>
+      </c>
+      <c r="S22" s="131">
+        <v>1</v>
+      </c>
+      <c r="T22" s="131">
+        <v>1</v>
+      </c>
       <c r="U22" s="137">
         <f t="shared" si="28"/>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="V22" s="131">
         <f t="shared" si="34"/>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="W22" s="137">
         <f t="shared" si="29"/>
         <v>13</v>
       </c>
       <c r="X22" s="131" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
       <c r="Y22" s="137">
         <f t="shared" si="30"/>
@@ -4456,7 +4486,7 @@
       </c>
       <c r="Z22" s="109">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>1430</v>
       </c>
       <c r="AA22" s="109">
         <f t="shared" si="32"/>
@@ -4464,7 +4494,7 @@
       </c>
       <c r="AB22" s="139">
         <f t="shared" si="35"/>
-        <v>-1430</v>
+        <v>0</v>
       </c>
       <c r="AC22" s="6"/>
       <c r="AF22" s="55"/>
@@ -5738,11 +5768,11 @@
       </c>
       <c r="U37" s="48">
         <f>SUM(U19:U36)</f>
-        <v>13</v>
+        <v>52</v>
       </c>
       <c r="V37" s="48">
         <f>SUM(V19:V36)</f>
-        <v>217</v>
+        <v>178</v>
       </c>
       <c r="W37" s="48">
         <f>SUM(W19:W36)</f>
@@ -5755,7 +5785,7 @@
       </c>
       <c r="Z37" s="70">
         <f t="shared" ref="Z37" si="38">tarif*U37</f>
-        <v>1430</v>
+        <v>5720</v>
       </c>
       <c r="AA37" s="70">
         <f t="shared" si="32"/>
@@ -5763,7 +5793,7 @@
       </c>
       <c r="AB37" s="70">
         <f t="shared" si="33"/>
-        <v>-23870</v>
+        <v>-19580</v>
       </c>
       <c r="AC37" s="50"/>
       <c r="AD37" s="37"/>
@@ -5796,8 +5826,8 @@
       <c r="J38" s="126"/>
       <c r="K38" s="77"/>
       <c r="L38" s="51"/>
-      <c r="M38" s="216"/>
-      <c r="N38" s="216"/>
+      <c r="M38" s="201"/>
+      <c r="N38" s="201"/>
       <c r="O38" s="140"/>
       <c r="P38" s="125"/>
       <c r="Q38" s="125"/>
@@ -6398,11 +6428,11 @@
       </c>
       <c r="U45" s="58">
         <f t="shared" si="51"/>
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="V45" s="58">
         <f t="shared" si="51"/>
-        <v>257</v>
+        <v>218</v>
       </c>
       <c r="W45" s="58">
         <f t="shared" si="51"/>
@@ -6415,7 +6445,7 @@
       </c>
       <c r="Z45" s="73">
         <f>Z11+Z17+Z37+Z43</f>
-        <v>8910</v>
+        <v>13200</v>
       </c>
       <c r="AA45" s="73">
         <f>AA11+AA17+AA37+AA43</f>
@@ -6423,7 +6453,7 @@
       </c>
       <c r="AB45" s="73">
         <f>Z45-K45</f>
-        <v>-28270</v>
+        <v>-23980</v>
       </c>
       <c r="AC45" s="63"/>
       <c r="AD45" s="28"/>
@@ -18301,11 +18331,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="M38:N38"/>
-    <mergeCell ref="P3:Y3"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="M18:N18"/>
     <mergeCell ref="AI17:AI20"/>
     <mergeCell ref="AE18:AH19"/>
     <mergeCell ref="B1:K1"/>
@@ -18317,6 +18342,11 @@
     <mergeCell ref="E3:J3"/>
     <mergeCell ref="M3:N3"/>
     <mergeCell ref="M12:N12"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="P3:Y3"/>
+    <mergeCell ref="B2:K2"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="M18:N18"/>
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="X6:X42">
@@ -18359,22 +18389,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="219" t="s">
+      <c r="A1" s="220" t="s">
         <v>93</v>
       </c>
-      <c r="B1" s="219"/>
-      <c r="C1" s="219"/>
-      <c r="D1" s="219"/>
-      <c r="E1" s="219"/>
+      <c r="B1" s="220"/>
+      <c r="C1" s="220"/>
+      <c r="D1" s="220"/>
+      <c r="E1" s="220"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="219" t="s">
+      <c r="A2" s="220" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="219"/>
-      <c r="C2" s="219"/>
-      <c r="D2" s="219"/>
-      <c r="E2" s="219"/>
+      <c r="B2" s="220"/>
+      <c r="C2" s="220"/>
+      <c r="D2" s="220"/>
+      <c r="E2" s="220"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -18406,22 +18436,22 @@
       <c r="A5" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="220" t="s">
+      <c r="B5" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="220" t="s">
+      <c r="C5" t="s">
         <v>121</v>
       </c>
-      <c r="D5" s="221">
+      <c r="D5" s="200">
         <v>46212</v>
       </c>
-      <c r="E5" s="220" t="s">
+      <c r="E5" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="220" t="s">
+      <c r="F5" t="s">
         <v>103</v>
       </c>
-      <c r="G5" s="220" t="s">
+      <c r="G5" t="s">
         <v>122</v>
       </c>
       <c r="I5" s="179" t="s">
@@ -18432,22 +18462,22 @@
       <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="220" t="s">
+      <c r="B6" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="220" t="s">
+      <c r="C6" t="s">
         <v>123</v>
       </c>
-      <c r="D6" s="221">
+      <c r="D6" s="200">
         <v>46208</v>
       </c>
-      <c r="E6" s="220" t="s">
+      <c r="E6" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="220" t="s">
+      <c r="F6" t="s">
         <v>103</v>
       </c>
-      <c r="G6" s="220" t="s">
+      <c r="G6" t="s">
         <v>124</v>
       </c>
       <c r="I6" s="144" t="s">
@@ -18504,26 +18534,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="219" t="s">
+      <c r="A1" s="220" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="219"/>
-      <c r="C1" s="219"/>
-      <c r="D1" s="219"/>
-      <c r="E1" s="219"/>
-      <c r="F1" s="219"/>
-      <c r="G1" s="219"/>
+      <c r="B1" s="220"/>
+      <c r="C1" s="220"/>
+      <c r="D1" s="220"/>
+      <c r="E1" s="220"/>
+      <c r="F1" s="220"/>
+      <c r="G1" s="220"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="219" t="s">
+      <c r="A2" s="220" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="219"/>
-      <c r="C2" s="219"/>
-      <c r="D2" s="219"/>
-      <c r="E2" s="219"/>
-      <c r="F2" s="219"/>
-      <c r="G2" s="219"/>
+      <c r="B2" s="220"/>
+      <c r="C2" s="220"/>
+      <c r="D2" s="220"/>
+      <c r="E2" s="220"/>
+      <c r="F2" s="220"/>
+      <c r="G2" s="220"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
@@ -18564,34 +18594,34 @@
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="222">
+      <c r="A5">
         <v>1</v>
       </c>
-      <c r="B5" s="222" t="s">
+      <c r="B5" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="222" t="s">
+      <c r="C5" t="s">
         <v>125</v>
       </c>
-      <c r="D5" s="222" t="s">
+      <c r="D5" t="s">
         <v>114</v>
       </c>
-      <c r="E5" s="222" t="s">
+      <c r="E5" t="s">
         <v>116</v>
       </c>
-      <c r="F5" s="224">
+      <c r="F5" s="200">
         <v>46189</v>
       </c>
-      <c r="G5" s="222" t="s">
+      <c r="G5" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="222" t="s">
+      <c r="H5" t="s">
         <v>101</v>
       </c>
-      <c r="I5" s="223" t="s">
+      <c r="I5" s="19" t="s">
         <v>126</v>
       </c>
-      <c r="J5" s="222" t="s">
+      <c r="J5" t="s">
         <v>127</v>
       </c>
       <c r="M5" s="182" t="s">
@@ -18602,34 +18632,34 @@
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="222">
+      <c r="A6">
         <v>2</v>
       </c>
-      <c r="B6" s="222" t="s">
+      <c r="B6" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="222" t="s">
+      <c r="C6" t="s">
         <v>128</v>
       </c>
-      <c r="D6" s="222" t="s">
+      <c r="D6" t="s">
         <v>116</v>
       </c>
-      <c r="E6" s="222" t="s">
+      <c r="E6" t="s">
         <v>114</v>
       </c>
-      <c r="F6" s="224">
+      <c r="F6" s="200">
         <v>46189</v>
       </c>
-      <c r="G6" s="222" t="s">
+      <c r="G6" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="222" t="s">
+      <c r="H6" t="s">
         <v>102</v>
       </c>
-      <c r="I6" s="223" t="s">
+      <c r="I6" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="J6" s="222" t="s">
+      <c r="J6" t="s">
         <v>130</v>
       </c>
       <c r="M6" s="183" t="s">
@@ -18640,34 +18670,34 @@
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="222">
+      <c r="A7">
         <v>3</v>
       </c>
-      <c r="B7" s="222" t="s">
+      <c r="B7" t="s">
         <v>131</v>
       </c>
-      <c r="C7" s="222" t="s">
+      <c r="C7" t="s">
         <v>132</v>
       </c>
-      <c r="D7" s="222" t="s">
+      <c r="D7" t="s">
         <v>114</v>
       </c>
-      <c r="E7" s="222" t="s">
+      <c r="E7" t="s">
         <v>114</v>
       </c>
-      <c r="F7" s="224">
+      <c r="F7" s="200">
         <v>46189</v>
       </c>
-      <c r="G7" s="222" t="s">
+      <c r="G7" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="222" t="s">
+      <c r="H7" t="s">
         <v>101</v>
       </c>
-      <c r="I7" s="223" t="s">
+      <c r="I7" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="J7" s="222" t="s">
+      <c r="J7" t="s">
         <v>134</v>
       </c>
       <c r="M7" s="184" t="s">
@@ -18678,34 +18708,34 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="222">
+      <c r="A8">
         <v>4</v>
       </c>
-      <c r="B8" s="222" t="s">
+      <c r="B8" t="s">
         <v>135</v>
       </c>
-      <c r="C8" s="222" t="s">
+      <c r="C8" t="s">
         <v>136</v>
       </c>
-      <c r="D8" s="222" t="s">
+      <c r="D8" t="s">
         <v>113</v>
       </c>
-      <c r="E8" s="222" t="s">
+      <c r="E8" t="s">
         <v>114</v>
       </c>
-      <c r="F8" s="224">
+      <c r="F8" s="200">
         <v>46189</v>
       </c>
-      <c r="G8" s="222" t="s">
+      <c r="G8" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="222" t="s">
+      <c r="H8" t="s">
         <v>101</v>
       </c>
-      <c r="I8" s="223" t="s">
+      <c r="I8" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="J8" s="222" t="s">
+      <c r="J8" t="s">
         <v>138</v>
       </c>
       <c r="M8" s="185" t="s">
@@ -18713,34 +18743,34 @@
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="222">
+      <c r="A9">
         <v>5</v>
       </c>
-      <c r="B9" s="222" t="s">
+      <c r="B9" t="s">
         <v>139</v>
       </c>
-      <c r="C9" s="222" t="s">
+      <c r="C9" t="s">
         <v>140</v>
       </c>
-      <c r="D9" s="222" t="s">
+      <c r="D9" t="s">
         <v>114</v>
       </c>
-      <c r="E9" s="222" t="s">
+      <c r="E9" t="s">
         <v>116</v>
       </c>
-      <c r="F9" s="224">
+      <c r="F9" s="200">
         <v>46189</v>
       </c>
-      <c r="G9" s="222" t="s">
+      <c r="G9" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="222" t="s">
+      <c r="H9" t="s">
         <v>115</v>
       </c>
-      <c r="I9" s="222" t="s">
+      <c r="I9" t="s">
         <v>141</v>
       </c>
-      <c r="J9" s="222" t="s">
+      <c r="J9" t="s">
         <v>142</v>
       </c>
     </row>

</xml_diff>